<commit_message>
adding the latest files
</commit_message>
<xml_diff>
--- a/dev_test/Diversification/Self Created Dataset/Manual Created Diversified Dataset/Disturbed Diversifications/Clinic_Visits/Clinic_Visits_original_0.xlsx
+++ b/dev_test/Diversification/Self Created Dataset/Manual Created Diversified Dataset/Disturbed Diversifications/Clinic_Visits/Clinic_Visits_original_0.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29616"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29621"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repo\table-diversification\dev_test\Diversification\Self Created Dataset\Manual Created Diversified Dataset\Disturbed Diversifications\Clinic_Visits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE8E3231-BE74-4F03-802E-1B13F0C759C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D6CBAFF-4233-4940-9177-6BFE39107433}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -612,6 +612,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">

</xml_diff>